<commit_message>
Rewrite Sugar News summary for 2026-08-18
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-18.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-18.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="140.05" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构下调食糖贸易、进口、出口或配额政策，相关数值为100%。进口、出口、关税或配额变化会改变国内外可用糖源和贸易流向。来源：Moneycontrol.com（https://www.moneycontrol.com/news/business/sugar-prices-hit-record-india-weighs-cutting-100-import-duty-14009062.html）。影响：利空糖价</t>
+          <t>印度政府据报正评估削减或取消100%食糖进口税，以应对国内糖价创新高并在节庆消费旺季前补充供应；APAC转载的同一事件称，马哈拉施特拉邦出厂糖价已升至约46卢比/公斤。若进口税下调落地，海外糖进入印度市场的成本会下降，国内可用糖源增加并压制印度现货糖价。政策仍处评估阶段，实际影响取决于进口窗口、配额和采购量。来源：Moneycontrol.com（https://www.moneycontrol.com/news/business/sugar-prices-hit-record-india-weighs-cutting-100-import-duty-14009062.html）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：进口政策放宽或进口量增加会补充国内可用糖源，对本地糖价形成压力。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="135.1" customHeight="1" s="2">
+          <t>利空：削减或取消100%进口税会降低进口糖到岸成本，补充印度国内可用糖源，并压制印度现货糖价；政策尚未最终落地。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="180" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -530,16 +530,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度糖厂下调糖厂运行和压榨安排，相关数值为15天。印度糖厂若增加开工或压榨，会加快当季食糖产出；若停产或延后开榨，则阶段性供应收紧。来源：ChiniMandi（https://www.chinimandi.com/maharashtra-starting-sugar-mills-15-days-early-could-cut-both-recovery-and-production/）。影响：利空糖价</t>
+          <t>印度中央政府考虑让糖厂较常规时间提前15天开榨，以缓解后期食糖短缺；但马哈拉施特拉糖业专家Vijay Autade认为，过早开榨可能使糖分回收率下降1-1.5个百分点，并造成每吨700-800卢比损失。回收率下降意味着同样甘蔗压榨量下食糖产出减少，若提前开榨反而压低产量，将加剧印度阶段性供应偏紧并支撑糖价。专家估计新季开榨时结转库存约400万吨，4-5万吨缺口可由11月底新糖供应弥补，因此短期影响取决于开榨时间是否真正提前。来源：ChiniMandi（https://www.chinimandi.com/maharashtra-starting-sugar-mills-15-days-early-could-cut-both-recovery-and-production/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利空：糖厂运行、压榨能力或原料供应改善会提高食糖生产节奏，增加阶段性供应。</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="129.05" customHeight="1" s="2">
+          <t>利多：提前15天开榨若导致糖分回收率下降1-1.5个百分点，会减少同等甘蔗压榨量对应的食糖产出，维持印度供应偏紧预期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="178.55" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -547,16 +547,16 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>印度糖业市场公布食糖价格和市场流通，糖价相关数值为Rs 60、Rs 65。印度价格上行通常会抬高补库成本，价格下行则说明供应压力或需求走弱正在传导到现货端。来源：ChiniMandi（https://www.chinimandi.com/punjab-wholesale-sugar-hits-record-rs-60-kg-retail-touches-rs-65/）。影响：中性</t>
+          <t>印度旁遮普邦批发市场糖价升至60卢比/公斤，零售价约65卢比/公斤；当地零售商称一周前零售价仍在54-56卢比/公斤，一个月前约46-48卢比/公斤。价格快速上涨且零售商反映正常供货不足，说明旁遮普市场出现阶段性供应紧张和囤货压力，对印度国内糖价形成支撑。邦食品部门要求经销商登记、申报库存并每周在食品库存监测门户更新，以限制囤货。来源：ChiniMandi（https://www.chinimandi.com/punjab-wholesale-sugar-hits-record-rs-60-kg-retail-touches-rs-65/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>中性：价格信息缺少明确涨跌幅或区域基准，暂不改变供需判断。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="136.75" customHeight="1" s="2">
+          <t>利多：旁遮普批发和零售糖价快速上涨，叠加供货不足和囤货压力，反映印度阶段性现货供应偏紧并支撑糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="173.6" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -564,16 +564,16 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>印度糖业市场公布食糖价格和市场流通，糖价相关数值为Rs 55。印度价格上行通常会抬高补库成本，价格下行则说明供应压力或需求走弱正在传导到现货端。来源：ChiniMandi（https://www.chinimandi.com/kolhapur-festive-demand-pushes-sugar-prices-higher-retail-rates-touch-rs-55-a-kilo/）。影响：利多糖价</t>
+          <t>印度科尔哈普尔糖厂因上一榨季产量低于预期、市场库存偏薄和节庆需求增加，将糖厂销售价推至4200-4500卢比/公担，零售价升至52-55卢比/公斤，高于政府3100卢比/公担的最低销售价。节庆消费抬升需求而库存偏薄，意味着贸易和零售端需要以更高价格补货，对印度现货糖价形成支撑。来源：ChiniMandi（https://www.chinimandi.com/kolhapur-festive-demand-pushes-sugar-prices-higher-retail-rates-touch-rs-55-a-kilo/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>利多：现货或出厂报价上涨反映阶段性供应偏紧或采购需求增强，会支撑短期糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="122.45" customHeight="1" s="2">
+          <t>利多：科尔哈普尔市场库存偏薄且节庆需求增加，推动糖厂销售价和零售价上行，支撑印度现货糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="180" customHeight="1" s="2">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -581,63 +581,46 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布甘蔗种植、蔗价或蔗农现金流，相关数值为58.31 lakh。甘蔗价格、面积或蔗款变化会影响蔗农种植意愿和下一季糖料供应。来源：ChiniMandi（https://www.chinimandi.com/sugarcane-area-under-kharif-2026-dips-to-58-31-lakh-hectares/）。影响：中性</t>
+          <t>印度农业与农民福利部数据显示，截至8月14日，2026年kharif季甘蔗种植面积为5831万公顷，低于去年同期5862万公顷，减少31万公顷；但仍高于2020/21-2024/25年度5420万公顷的正常面积。甘蔗面积同比小幅下降会削弱部分地区下一季糖料供应预期，但全国面积仍高于正常水平，且北方邦和哈里亚纳面积分别增加36万和11万公顷，对糖价影响偏中性。马哈拉施特拉和旁遮普面积各减少14万公顷，后续仍需看单产和出糖率是否同步下降。来源：ChiniMandi（https://www.chinimandi.com/sugarcane-area-under-kharif-2026-dips-to-58-31-lakh-hectares/）。影响：中性</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>中性：原文只说明甘蔗生产或蔗农经营变化，尚未给出可判断糖料供应增减的明确方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="115.3" customHeight="1" s="2">
+          <t>中性：印度甘蔗面积同比减少31万公顷会削弱部分地区糖料供应预期，但全国面积仍高于正常水平且主产区增减分化，暂不足以单独改变糖价方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="118.6" customHeight="1" s="2">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布食糖贸易、进口、出口或配额政策，相关数值为100%。进口、出口、关税或配额变化会改变国内外可用糖源和贸易流向。来源：APAC Media（https://apacnewsnetwork.com/2026/08/india-sugar-import-duty-cut-record-prices/）。影响：利空糖价</t>
+          <t>泰国气象局预报（2026-08-18），乌隆他尼、加拉信、北碧、沙缴等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>利空：进口政策放宽或进口量增加会补充国内可用糖源，对本地糖价形成压力。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118.6" customHeight="1" s="2">
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="170.3" customHeight="1" s="2">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>尼泊尔</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>泰国气象局预报（2026-08-18），乌隆他尼、加拉信、北碧、沙缴等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
+          <t>尼泊尔食糖价格在节日前由95-100卢比/公斤升至约120卢比/公斤，零售端报告缺货；当地节日期间食糖消费预计较平时翻倍，而政府进口安排尚未最终确定。国内库存下降和进口决策延迟会收紧尼泊尔市场可用糖源，推高当地糖价并增加后续进口需求。若进口审批继续推迟，节前囤货可能进一步放大局部短缺。来源：ChiniMandi（https://www.chinimandi.com/nepal-sugar-price-hits-rs-120-per-kg-ahead-of-festival-as-shortage-looms/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="131.8" customHeight="1" s="2">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>尼泊尔</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>尼泊尔糖业市场公布食糖价格和市场流通，糖价相关数值为Rs 120。尼泊尔价格上行通常会抬高补库成本，价格下行则说明供应压力或需求走弱正在传导到现货端。来源：ChiniMandi（https://www.chinimandi.com/nepal-sugar-price-hits-rs-120-per-kg-ahead-of-festival-as-shortage-looms/）。影响：中性</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>中性：价格信息缺少明确涨跌幅或区域基准，暂不改变供需判断。</t>
+          <t>利多：尼泊尔库存下降、进口安排延迟和节日消费翻倍会收紧当地可用糖源，推高尼泊尔糖价并增加进口需求。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Sugar News Brazil hedge and India logic
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-18.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-18.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -508,17 +508,17 @@
     <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>巴西</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度政府据报正评估削减或取消100%食糖进口税，以应对国内糖价创新高并在节庆消费旺季前补充供应；APAC转载的同一事件称，马哈拉施特拉邦出厂糖价已升至约46卢比/公斤。若进口税下调落地，海外糖进入印度市场的成本会下降，国内可用糖源增加并压制印度现货糖价。政策仍处评估阶段，实际影响取决于进口窗口、配额和采购量。来源：Moneycontrol.com（https://www.moneycontrol.com/news/business/sugar-prices-hit-record-india-weighs-cutting-100-import-duty-14009062.html）。影响：利空糖价</t>
+          <t>近期重要消息：Hedgepoint在7月28日的2026/27巴西中南部报告中维持甘蔗压榨量6.35亿吨、制糖比约47.3%的预测，并指出相当一部分未来食糖产量已通过国际期货套保和长期出口合同锁定。套保和长协限制糖厂在油价或乙醇经济性改善时迅速把甘蔗转向乙醇，同时减少未锁定糖源的机动空间；在北半球可出口供应下调的背景下，这会支撑远月原糖价格。该来源没有披露具体套保比例，后续若Datagro、Archer、StoneX、Hedgepoint或Reuters更新比例，需要列为巴西重点观察。来源：Hedgepoint Global Markets（https://hedgepointglobal.com/en/blog/safra-de-cana-2026/27-a-din%C3%A2mica-do-mix-de-produ%C3%A7%C3%A3o-frente-ao-cen%C3%A1rio-energ%C3%A9tico-global）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：削减或取消100%进口税会降低进口糖到岸成本，补充印度国内可用糖源，并压制印度现货糖价；政策尚未最终落地。</t>
+          <t>利多：巴西未来食糖产量已有相当一部分通过期货套保和长期出口合同锁定，说明可机动供应减少并支撑远月原糖价格；但来源未给出具体套保比例，后续比例数据需要单独核对。</t>
         </is>
       </c>
     </row>
@@ -530,95 +530,112 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
+          <t>印度政府据报正评估削减或取消100%食糖进口税，以应对国内糖价创纪录并在节庆消费旺季前补充供应；APAC转载的同一事件称，马哈拉施特拉邦出厂糖价已升至约46卢比/公斤。进口税调整讨论本身说明印度国内糖源偏紧、价格已高到需要引入海外糖源，短期强化供应紧张预期并利多糖价；若政策最终落地并形成实际进口，后续才会增加国内供应、压制印度现货糖价。来源：Moneycontrol.com（https://www.moneycontrol.com/news/business/sugar-prices-hit-record-india-weighs-cutting-100-import-duty-14009062.html）。影响：利多糖价</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>利多：印度评估削减或取消100%进口税是国内糖价创纪录、节前可用糖源紧张的政策信号，短期强化供应偏紧预期；若进口真正落地，后续才会增加供应并压制现货。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="180" customHeight="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>印度中央政府考虑让糖厂较常规时间提前15天开榨，以缓解后期食糖短缺；但马哈拉施特拉糖业专家Vijay Autade认为，过早开榨可能使糖分回收率下降1-1.5个百分点，并造成每吨700-800卢比损失。回收率下降意味着同样甘蔗压榨量下食糖产出减少，若提前开榨反而压低产量，将加剧印度阶段性供应偏紧并支撑糖价。专家估计新季开榨时结转库存约400万吨，4-5万吨缺口可由11月底新糖供应弥补，因此短期影响取决于开榨时间是否真正提前。来源：ChiniMandi（https://www.chinimandi.com/maharashtra-starting-sugar-mills-15-days-early-could-cut-both-recovery-and-production/）。影响：利多糖价</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>利多：提前15天开榨若导致糖分回收率下降1-1.5个百分点，会减少同等甘蔗压榨量对应的食糖产出，维持印度供应偏紧预期。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="178.55" customHeight="1" s="2">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="178.55" customHeight="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>印度旁遮普邦批发市场糖价升至60卢比/公斤，零售价约65卢比/公斤；当地零售商称一周前零售价仍在54-56卢比/公斤，一个月前约46-48卢比/公斤。价格快速上涨且零售商反映正常供货不足，说明旁遮普市场出现阶段性供应紧张和囤货压力，对印度国内糖价形成支撑。邦食品部门要求经销商登记、申报库存并每周在食品库存监测门户更新，以限制囤货。来源：ChiniMandi（https://www.chinimandi.com/punjab-wholesale-sugar-hits-record-rs-60-kg-retail-touches-rs-65/）。影响：利多糖价</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>利多：旁遮普批发和零售糖价快速上涨，叠加供货不足和囤货压力，反映印度阶段性现货供应偏紧并支撑糖价。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="173.6" customHeight="1" s="2">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="173.6" customHeight="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>印度科尔哈普尔糖厂因上一榨季产量低于预期、市场库存偏薄和节庆需求增加，将糖厂销售价推至4200-4500卢比/公担，零售价升至52-55卢比/公斤，高于政府3100卢比/公担的最低销售价。节庆消费抬升需求而库存偏薄，意味着贸易和零售端需要以更高价格补货，对印度现货糖价形成支撑。来源：ChiniMandi（https://www.chinimandi.com/kolhapur-festive-demand-pushes-sugar-prices-higher-retail-rates-touch-rs-55-a-kilo/）。影响：利多糖价</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>利多：科尔哈普尔市场库存偏薄且节庆需求增加，推动糖厂销售价和零售价上行，支撑印度现货糖价。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="180" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7" ht="180" customHeight="1" s="2">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>印度</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>印度农业与农民福利部数据显示，截至8月14日，2026年kharif季甘蔗种植面积为5831万公顷，低于去年同期5862万公顷，减少31万公顷；但仍高于2020/21-2024/25年度5420万公顷的正常面积。甘蔗面积同比小幅下降会削弱部分地区下一季糖料供应预期，但全国面积仍高于正常水平，且北方邦和哈里亚纳面积分别增加36万和11万公顷，对糖价影响偏中性。马哈拉施特拉和旁遮普面积各减少14万公顷，后续仍需看单产和出糖率是否同步下降。来源：ChiniMandi（https://www.chinimandi.com/sugarcane-area-under-kharif-2026-dips-to-58-31-lakh-hectares/）。影响：中性</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>中性：印度甘蔗面积同比减少31万公顷会削弱部分地区糖料供应预期，但全国面积仍高于正常水平且主产区增减分化，暂不足以单独改变糖价方向。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118.6" customHeight="1" s="2">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>印度农业与农民福利部数据显示，截至8月14日，2026年kharif季甘蔗种植面积为5831万公顷，低于去年同期5862万公顷、减少31万公顷，但仍高于2020/21-2024/25年度5420万公顷的正常面积，且北方邦和哈里亚纳面积分别增加36万和11万公顷。全国面积高于正常水平、北方邦等主产区扩种提高下一季糖料供应预期，对糖价偏利空；马哈拉施特拉和旁遮普各减少14万公顷，只削弱利空幅度而不改变“面积增加对应供应压力”的判断。来源：ChiniMandi（https://www.chinimandi.com/sugarcane-area-under-kharif-2026-dips-to-58-31-lakh-hectares/）。影响：利空糖价</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>利空：印度甘蔗面积仍高于正常水平，且北方邦、哈里亚纳面积增加，提高下一季糖料和食糖供应预期；同比小降及马哈拉施特拉、旁遮普减少只削弱利空幅度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="118.6" customHeight="1" s="2">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>泰国气象局预报（2026-08-18），乌隆他尼、加拉信、北碧、沙缴等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="170.3" customHeight="1" s="2">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="170.3" customHeight="1" s="2">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>尼泊尔</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>尼泊尔食糖价格在节日前由95-100卢比/公斤升至约120卢比/公斤，零售端报告缺货；当地节日期间食糖消费预计较平时翻倍，而政府进口安排尚未最终确定。国内库存下降和进口决策延迟会收紧尼泊尔市场可用糖源，推高当地糖价并增加后续进口需求。若进口审批继续推迟，节前囤货可能进一步放大局部短缺。来源：ChiniMandi（https://www.chinimandi.com/nepal-sugar-price-hits-rs-120-per-kg-ahead-of-festival-as-shortage-looms/）。影响：利多糖价</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>利多：尼泊尔库存下降、进口安排延迟和节日消费翻倍会收紧当地可用糖源，推高尼泊尔糖价并增加进口需求。</t>
         </is>

</xml_diff>